<commit_message>
Template page and sign-ups: money.flowlytix.co/template, owner list in Setup
- template.html: EN/TH landing page in the /pro style, pictures of the real
  template (sample figures only), email form with a separate unticked news
  box, hidden bot field and privacy note; download button straight after.
  Meta Lead + GA4 generate_lead once per browser, never the email.
- worker/leads.js: POST /api/template/lead into SURVEY_DB (table
  template_leads, one row per email), rate limit LEAD_LIMIT (5/min per
  connection and per email); owner-only list, CSV and delete.
- App: Setup > Template sign-ups (count, news OK, last 7 days, list,
  Download CSV, two-tap Delete), with a ? tip and Thai.
- Template: a little space before the month so amount and month don't touch.
- 18 new worker tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrYSikNGDHCJsHD7QUpoxC
</commit_message>
<xml_diff>
--- a/templates/flowlytix-yearly-bills.xlsx
+++ b/templates/flowlytix-yearly-bills.xlsx
@@ -216,7 +216,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
+      <alignment vertical="center" horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -225,7 +225,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
+      <alignment vertical="center" horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>

</xml_diff>

<commit_message>
Import from my template: bring the filled-in yearly bills template into the plan
- Setup > Import from my template: choose the .xlsx or .csv; it is read in the
  browser only (plain code, the browser's own unzip), never sent to our server.
  Preview first: ready / needs fixing with a plain reason / already in your
  plan / sample rows skipped. New categories get the group the person picks.
  Add = same as + Add item; nothing existing is changed or deleted; free plan.
- Welcome screen: "import my template next" tick; /?import=template (the
  template page's next step) opens Setup at the import.
- ? tip, Setup tour step, How to use entry, Thai for every line.
- Template: Read me step 6 (import into Money); /template next step = import.
- tests/import.test.mjs (29 checks) with a fixture re-saved by LibreOffice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrYSikNGDHCJsHD7QUpoxC
</commit_message>
<xml_diff>
--- a/templates/flowlytix-yearly-bills.xlsx
+++ b/templates/flowlytix-yearly-bills.xlsx
@@ -425,115 +425,129 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="5" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.  Use Flowlytix Money? In the app, Setup › Import from my template adds these bills to your plan in one step (keep the columns in this order).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Tip: add regular costs like food and transport too, so the totals compare fairly with your pay.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="4"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="B14" s="3" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Want to know how much to set aside each month so every bill is covered? Try Flowlytix Money, Pro free for 30 days, no card needed.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="7" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">→  money.flowlytix.co/pro</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="5" t="inlineStr">
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">This file stays on your computer. Flowlytix never sees what you type in it.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="2" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">วิธีใช้</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="20" ht="36" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">1.  แท็บ Bills: ใส่บิลหรือค่าใช้จ่ายประจำแถวละ 1 รายการ (ค่าเช่า ค่าอาหาร ประกัน ค่าเทอม ภาษีรถ ทริปเที่ยว) แถวสีเทา 5 แถวเป็นตัวอย่าง ลบทิ้งหรือพิมพ์ทับได้เลย</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
+    <row r="21" ht="52" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">2.  ความถี่ (How often): เลือกจากรายการ (รายเดือน รายไตรมาส ปีละสองครั้ง รายปี ครั้งเดียว) เดือนที่ครบกำหนดครั้งแรก = เดือนที่ต้องจ่ายงวดถัดไป เช่น Mar 2027 (รายเดือนเว้นว่างได้) เดือนสิ้นสุดใส่เฉพาะรายการที่จะหมด เช่น งวดสุดท้ายของเงินกู้</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="36" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">3.  หมวด (Category): พิมพ์คำของคุณเอง หรือใช้หมวดของ Flowlytix Money: Food (อาหาร), Transport (การเดินทาง), Bills (บิล), Phone &amp; internet, Sinking fund (กองทุนสะสม), Shopping, Family (ครอบครัว)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">4.  แท็บ Income: รายได้สุทธิแต่ละเดือน (เงินที่เข้าบัญชีจริง)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="24" ht="36" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">5.  แท็บ Year view: เลือกเดือนเริ่มต้น แล้วดูบิลที่ต้องจ่ายแต่ละเดือนเทียบกับรายได้ แถวสีแดง = เดือนนั้นบิลมากกว่ารายได้</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="5" t="inlineStr">
+    <row r="25" ht="36" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.  ใช้ Flowlytix Money? ในแอป ไปที่ ตั้งค่า › นำเข้าจากเทมเพลตของฉัน เพื่อเพิ่มบิลเหล่านี้เข้าแผนในขั้นตอนเดียว (อย่าสลับลำดับคอลัมน์)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">เคล็ดลับ: ใส่ค่าใช้จ่ายประจำอย่างค่าอาหารและค่าเดินทางด้วย ยอดรวมจะเทียบกับรายได้ได้ตรงขึ้น</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="B26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="4"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">อยากรู้ว่าแต่ละเดือนต้องกันเงินไว้เท่าไร ให้มีพอจ่ายทุกบิล? ลองใช้ Flowlytix Money ใช้ Pro ฟรี 30 วัน ไม่ต้องใช้บัตร</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="7" t="inlineStr">
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">→  money.flowlytix.co/pro</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="5" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">ไฟล์นี้อยู่ในเครื่องของคุณเท่านั้น Flowlytix ไม่เห็นข้อมูลที่คุณกรอก</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="28">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
@@ -560,10 +574,12 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B15" r:id="rId1"/>
-    <hyperlink ref="B27" r:id="rId2"/>
+    <hyperlink ref="B16" r:id="rId1"/>
+    <hyperlink ref="B29" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>